<commit_message>
feat: Update max_tokens in config and enhance LLMClient for OpenAI models
</commit_message>
<xml_diff>
--- a/output/classified_messages.xlsx
+++ b/output/classified_messages.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Priority</t>
         </is>
       </c>
     </row>
@@ -436,7 +446,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>District: Colombo | Intent: Info | Priority: High</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -448,7 +468,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Rescue | Priority: High</t>
+          <t>Gampaha</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -460,7 +490,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>District: Kandy | Intent: Info | Priority: Low</t>
+          <t>Kandy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -472,7 +512,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Supply | Priority: High</t>
+          <t>Gampaha</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -484,7 +534,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>District: Colombo | Intent: Info | Priority: Low</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -496,7 +556,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>District: None | Intent: Rescue | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -508,7 +578,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Info | Priority: Low</t>
+          <t>Gampaha</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -520,7 +600,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>District: None | Intent: Rescue | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -532,7 +622,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -544,7 +644,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>District: None | Intent: Info | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -556,7 +666,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>District: Badulla | Intent: Rescue | Priority: High</t>
+          <t>Badulla</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -568,7 +688,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -580,7 +710,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>District: Colombo | Intent: Info | Priority: Low</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -592,7 +732,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>District: Kolonnawa | Intent: Rescue | Priority: High</t>
+          <t>Kolonnawa</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -604,7 +754,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>District: None | Intent: Info | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -616,7 +776,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Supply | Priority: High</t>
+          <t>Gampaha</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -628,7 +798,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>District: Kitulgala | Intent: Rescue | Priority: High</t>
+          <t>Kitulgala</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -640,7 +820,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>District: None | Intent: Info | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -652,7 +842,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>District: None | Intent: Info | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -664,7 +864,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -676,7 +886,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>District: Kaduwela | Intent: Rescue | Priority: High</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -688,7 +908,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -700,7 +930,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>District: None | Intent: Supply | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -712,7 +952,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>District: Colombo | Intent: Info | Priority: Low</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -724,7 +974,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>District: Colombo | Intent: Rescue | Priority: High</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -736,7 +996,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>District: Matara | Intent: Info | Priority: Low</t>
+          <t>Matara</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -748,7 +1018,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>District: Kalutara | Intent: Info | Priority: High</t>
+          <t>Kalutara</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -760,7 +1040,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>District: Ja-Ela | Intent: Rescue | Priority: High</t>
+          <t>Ja-Ela</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -772,7 +1062,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>District: Galle | Intent: Info | Priority: Low</t>
+          <t>Galle</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -784,7 +1084,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>District: Ratnapura | Intent: Info | Priority: Low</t>
+          <t>Ratnapura</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -796,7 +1106,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Rescue | Priority: High</t>
+          <t>Wellampitiya</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -808,7 +1128,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>District: Galle | Intent: Other | Priority: Low</t>
+          <t>Galle</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -820,7 +1150,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>District: None | Intent: Supply | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -832,7 +1172,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>District: Nuwara Eliya | Intent: Info | Priority: Low</t>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -844,7 +1194,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Rescue | Priority: High</t>
+          <t>Gampaha</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -856,7 +1216,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -868,7 +1238,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>District: Colombo | Intent: Info | Priority: Low</t>
+          <t>Colombo</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -880,7 +1260,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -892,7 +1282,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>District: Kegalle | Intent: Info | Priority: High</t>
+          <t>Kegalle</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -904,7 +1304,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>District: None | Intent: Supply | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -916,7 +1326,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>District: Gampaha | Intent: Rescue | Priority: High</t>
+          <t>Gampaha</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -928,7 +1348,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>District: None | Intent: Rescue | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -940,7 +1370,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>District: None | Intent: Other | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -952,7 +1392,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>District: Kandy | Intent: Rescue | Priority: High</t>
+          <t>Kandy</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -964,7 +1414,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>District: Kandy | Intent: Info | Priority: Low</t>
+          <t>Kandy</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -976,7 +1436,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>District: None | Intent: Info | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -988,7 +1458,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>District: None | Intent: Supply | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1480,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>District: None | Intent: Rescue | Priority: High</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Rescue</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1502,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>District: None | Intent: Supply | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1524,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>District: None | Intent: Info | Priority: Low</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add district classification to config and enhance classifier logic
</commit_message>
<xml_diff>
--- a/output/classified_messages.xlsx
+++ b/output/classified_messages.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kolonnawa</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kitulgala</t>
+          <t>Kandy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ja-Ela</t>
+          <t>Gampaha</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wellampitiya</t>
+          <t>Kandy</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1353,12 +1353,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rescue</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>